<commit_message>
feat(tests): use cached FMR dissemination schema for final validation
Replace the self-generated dissemination schema with a pre-existing
one fetched from FMR (WB.GGH.HSP:DS_ASPIRE), cached as a pickle
fixture. This makes Step 6 validation meaningful — it validates
against an independent schema rather than one derived from the output.

Tests that depend on the schema cache skip gracefully when the cache
file (tests/fixtures/cassettes/pipeline_dis_schema.pkl) is absent.

To generate the cache, run:
  client = px.api.fmr.RegistryClient(fmr_url)
  schema = client.get_schema("datastructure", agency="WB.GGH.HSP",
                             id="DS_ASPIRE", version="1.0.0")
  pickle.dump(schema, open("pipeline_dis_schema.pkl", "wb"))

https://claude.ai/code/session_01CwNPbbnSksjkKYW3S3A92V
</commit_message>
<xml_diff>
--- a/tests/fixtures/data/pipeline_mapping_template.xlsx
+++ b/tests/fixtures/data/pipeline_mapping_template.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TEST.AGENCY</t>
+          <t>WB.GGH.HSP</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TEST.AGENCY:DS_TEST(1.0.0)</t>
+          <t>WB.GGH.HSP:DS_ASPIRE(1.0.0)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(tests): validate against real DS_ASPIRE dissemination schema
Update raw data and mapping template to use valid DS_ASPIRE codelist
values (SPL_TR_AMT_RD indicator, proper fixed values for all mandatory
dimensions). Step 6 now validates the pipeline output against the real
FMR-cached dissemination schema, catching missing columns, invalid
codelist values, and schema mismatches.

https://claude.ai/code/session_01CwNPbbnSksjkKYW3S3A92V
</commit_message>
<xml_diff>
--- a/tests/fixtures/data/pipeline_mapping_template.xlsx
+++ b/tests/fixtures/data/pipeline_mapping_template.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,26 +575,31 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VALUE</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FREQ</t>
+          <t>OBS_VALUE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>fixed:A</t>
+          <t>implicit</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VALUE</t>
+          <t>TIME_PERIOD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OBS_VALUE</t>
+          <t>TIME_PERIOD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -604,19 +609,98 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>TIME_PERIOD</t>
-        </is>
-      </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TIME_PERIOD</t>
+          <t>FREQ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>implicit</t>
+          <t>fixed:A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fixed:_T</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>URBANIZATION</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fixed:_T</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PROGRAM_TYPE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fixed:_Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BENEFICIARY_TYPE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fixed:DI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>INCOME_GROUP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>fixed:_T</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PRET</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>fixed:_Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>UNIT_MEASURE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>fixed:U</t>
         </is>
       </c>
     </row>
@@ -649,12 +733,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SPL_COV_TOT</t>
+          <t>SPL_TR_AMT_RD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TEST_PIPELINE_SPL_COV_TOT</t>
+          <t>SPL_TR_AMT_RD</t>
         </is>
       </c>
     </row>

</xml_diff>